<commit_message>
Remove perpetuity instruction from lesson 3 workbook
</commit_message>
<xml_diff>
--- a/lessons/03/files/ファイナンス入門演習_第3回.xlsx
+++ b/lessons/03/files/ファイナンス入門演習_第3回.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PV関数" sheetId="1" r:id="R7e844588bbb8453c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="練習1" sheetId="2" r:id="Rf958f1b21352453e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="練習2" sheetId="3" r:id="R39115fe000a74d76"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="練習3" sheetId="4" r:id="Ref3019e20cdc409e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="練習4" sheetId="5" r:id="Re0ca45fd780e43b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="練習5" sheetId="6" r:id="R3ed6c610870e4f43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="練習6" sheetId="7" r:id="R2bdab914e7fe4c90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PV関数" sheetId="1" r:id="Rfd0605bf2e9f4e1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="練習1" sheetId="2" r:id="R923bb7dddf334605"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="練習2" sheetId="3" r:id="R4be08444c72b4cff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="練習3" sheetId="4" r:id="R85c6d19032644d7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="練習4" sheetId="5" r:id="R560b3429ef284e38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="練習5" sheetId="6" r:id="R67bceb4f8cf14d6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="練習6" sheetId="7" r:id="R299667561eae4395"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3106,9 +3106,7 @@
     </x:row>
     <x:row r="24" ht="36" customHeight="1">
       <x:c r="A24" s="3"/>
-      <x:c r="B24" s="4" t="str">
-        <x:v>永久年金では r &gt; 0 とします。期間数を大きくしたPV関数で代用せず、CF/r を使います。</x:v>
-      </x:c>
+      <x:c r="B24" s="4" t="str"/>
       <x:c r="C24" s="4"/>
       <x:c r="D24" s="4"/>
       <x:c r="E24" s="4"/>
@@ -3494,9 +3492,7 @@
     </x:row>
     <x:row r="24" ht="36" customHeight="1">
       <x:c r="A24" s="3"/>
-      <x:c r="B24" s="4" t="str">
-        <x:v>永久年金では r &gt; 0 とします。期間数を大きくしたPV関数で代用せず、CF/r を使います。</x:v>
-      </x:c>
+      <x:c r="B24" s="4" t="str"/>
       <x:c r="C24" s="4"/>
       <x:c r="D24" s="4"/>
       <x:c r="E24" s="4"/>

</xml_diff>